<commit_message>
table for nonterm in TPDB_NO
</commit_message>
<xml_diff>
--- a/TPDB_NO/analysis_for_TPDB_NO.xlsx
+++ b/TPDB_NO/analysis_for_TPDB_NO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\repo\TerminationDatabase\TPDB_NO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BCA3C33-BAA0-45DD-B05E-A173FAD7615A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6891A45-A5A9-41C5-9B3D-11164D92EA56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9171" yWindow="0" windowWidth="9429" windowHeight="11709" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -447,19 +447,21 @@
         <v>3</v>
       </c>
       <c r="C3">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="D3">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F3">
-        <v>89</v>
+        <f>C3+D3+E3</f>
+        <v>76</v>
       </c>
       <c r="G3">
-        <v>5.35</v>
+        <f>(24*5.36+6*6.13+46*5.1)/(24+6+46)</f>
+        <v>5.2634210526315783</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.35">
@@ -467,19 +469,21 @@
         <v>1</v>
       </c>
       <c r="C4">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="D4">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E4">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F4">
-        <v>68</v>
+        <f t="shared" ref="F4:F5" si="0">C4+D4+E4</f>
+        <v>60</v>
       </c>
       <c r="G4">
-        <v>0.91</v>
+        <f>(17*0.9+8*0.91+35*0.94)/60</f>
+        <v>0.92466666666666675</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.35">
@@ -487,19 +491,21 @@
         <v>2</v>
       </c>
       <c r="C5">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="D5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E5">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F5">
-        <v>89</v>
+        <f t="shared" si="0"/>
+        <v>58</v>
       </c>
       <c r="G5">
-        <v>10.79</v>
+        <f>(25*9.94+3*16.33+30*10.31)/58</f>
+        <v>10.461896551724138</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.35">
@@ -516,6 +522,7 @@
         <v>18</v>
       </c>
       <c r="F6">
+        <f>C6+D6+E6</f>
         <v>110</v>
       </c>
     </row>

</xml_diff>